<commit_message>
se agrega archivo de configuracion y ajustes visuales
</commit_message>
<xml_diff>
--- a/datos_prueba/master_league_ejemplo.xlsx
+++ b/datos_prueba/master_league_ejemplo.xlsx
@@ -8,6 +8,7 @@
     <sheet state="visible" name="Equipos" sheetId="3" r:id="rId6"/>
     <sheet state="visible" name="Eventos" sheetId="4" r:id="rId7"/>
     <sheet state="visible" name="Fixture" sheetId="5" r:id="rId8"/>
+    <sheet state="visible" name="Configuraciones" sheetId="6" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -15,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4178" uniqueCount="1159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4188" uniqueCount="1168">
   <si>
     <t xml:space="preserve">id</t>
   </si>
@@ -3492,6 +3493,34 @@
   </si>
   <si>
     <t xml:space="preserve">2027-06-14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">key</t>
+  </si>
+  <si>
+    <t xml:space="preserve">value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://mrrichar.netlify.app/logo.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">appTitle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MRRICHAR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">splashTitle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Liga Master
+MRRICHAR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">splashSubtitle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tu liga de fútbol profesional personalizada</t>
   </si>
 </sst>
 </file>
@@ -16950,4 +16979,53 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>1159</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1160</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="s">
+        <v>931</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>1161</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="s">
+        <v>1162</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>1163</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="s">
+        <v>1164</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>1165</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="s">
+        <v>1166</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>1167</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
se agrega version configurable desde excel en pantalla de carga
</commit_message>
<xml_diff>
--- a/datos_prueba/master_league_ejemplo.xlsx
+++ b/datos_prueba/master_league_ejemplo.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4188" uniqueCount="1168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4190" uniqueCount="1170">
   <si>
     <t xml:space="preserve">id</t>
   </si>
@@ -3521,6 +3521,12 @@
   </si>
   <si>
     <t xml:space="preserve">Tu liga de fútbol profesional personalizada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">version</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.0.6+8</t>
   </si>
 </sst>
 </file>
@@ -17025,6 +17031,14 @@
         <v>1167</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="1" t="s">
+        <v>1168</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>1169</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
se ajusta logo pantalla carga y se cambia origen de logo pantalla inicio
</commit_message>
<xml_diff>
--- a/datos_prueba/master_league_ejemplo.xlsx
+++ b/datos_prueba/master_league_ejemplo.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4190" uniqueCount="1170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4192" uniqueCount="1172">
   <si>
     <t xml:space="preserve">id</t>
   </si>
@@ -3502,6 +3502,12 @@
   </si>
   <si>
     <t xml:space="preserve">https://mrrichar.netlify.app/logo.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">homeLogoUrl</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://mrrichar.netlify.app/Logo%20Liga%20Master_.png</t>
   </si>
   <si>
     <t xml:space="preserve">appTitle</t>
@@ -3526,7 +3532,7 @@
     <t xml:space="preserve">version</t>
   </si>
   <si>
-    <t xml:space="preserve">1.0.7+9</t>
+    <t xml:space="preserve">1.0.8+10</t>
   </si>
 </sst>
 </file>
@@ -17039,6 +17045,14 @@
         <v>1169</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="1" t="s">
+        <v>1170</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>1171</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>